<commit_message>
a tot of small changes in paper text
</commit_message>
<xml_diff>
--- a/Data/KW_dunn_between_month.xlsx
+++ b/Data/KW_dunn_between_month.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yaroslav\OneDrive\Рабочий стол\Python_repos\Python_projects_ICG_SB_RAS\Four_host_species_OF\Data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF730FCA-C22C-4E4E-96DD-0DE1519966D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="KW_dunn_between_month" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -109,8 +115,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -158,7 +164,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -181,11 +187,106 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -194,19 +295,45 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -244,7 +371,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -278,6 +405,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -312,9 +440,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -487,11 +616,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S52"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:T52"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:19">
+    <row r="1" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -505,7 +634,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:19">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -519,7 +648,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:19">
+    <row r="3" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -533,7 +662,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:19">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>0</v>
       </c>
@@ -571,7 +700,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:19">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -579,10 +708,10 @@
         <v>1</v>
       </c>
       <c r="C5" s="4">
-        <v>0.164</v>
+        <v>0.16400000000000001</v>
       </c>
       <c r="D5" s="4">
-        <v>0.164</v>
+        <v>0.16400000000000001</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>0</v>
@@ -591,10 +720,10 @@
         <v>1</v>
       </c>
       <c r="H5" s="4">
-        <v>0.358</v>
+        <v>0.35799999999999998</v>
       </c>
       <c r="I5" s="5">
-        <v>0.043</v>
+        <v>4.2999999999999997E-2</v>
       </c>
       <c r="K5" s="3" t="s">
         <v>0</v>
@@ -603,10 +732,10 @@
         <v>1</v>
       </c>
       <c r="M5" s="4">
-        <v>0.722</v>
+        <v>0.72199999999999998</v>
       </c>
       <c r="N5" s="4">
-        <v>0.059</v>
+        <v>5.8999999999999997E-2</v>
       </c>
       <c r="P5" s="3" t="s">
         <v>0</v>
@@ -615,18 +744,18 @@
         <v>1</v>
       </c>
       <c r="R5" s="4">
-        <v>0.288</v>
+        <v>0.28799999999999998</v>
       </c>
       <c r="S5" s="5">
-        <v>0.051</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19">
+        <v>5.0999999999999997E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B6" s="4">
-        <v>0.164</v>
+        <v>0.16400000000000001</v>
       </c>
       <c r="C6" s="4">
         <v>1</v>
@@ -638,45 +767,45 @@
         <v>1</v>
       </c>
       <c r="G6" s="4">
-        <v>0.358</v>
+        <v>0.35799999999999998</v>
       </c>
       <c r="H6" s="4">
         <v>1</v>
       </c>
       <c r="I6" s="5">
-        <v>0.006</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="K6" s="3" t="s">
         <v>1</v>
       </c>
       <c r="L6" s="4">
-        <v>0.722</v>
+        <v>0.72199999999999998</v>
       </c>
       <c r="M6" s="4">
         <v>1</v>
       </c>
       <c r="N6" s="5">
-        <v>0.047</v>
+        <v>4.7E-2</v>
       </c>
       <c r="P6" s="3" t="s">
         <v>1</v>
       </c>
       <c r="Q6" s="4">
-        <v>0.288</v>
+        <v>0.28799999999999998</v>
       </c>
       <c r="R6" s="4">
         <v>1</v>
       </c>
       <c r="S6" s="5">
-        <v>0.004</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19">
+        <v>4.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B7" s="4">
-        <v>0.164</v>
+        <v>0.16400000000000001</v>
       </c>
       <c r="C7" s="4">
         <v>0.749</v>
@@ -688,10 +817,10 @@
         <v>2</v>
       </c>
       <c r="G7" s="5">
-        <v>0.043</v>
+        <v>4.2999999999999997E-2</v>
       </c>
       <c r="H7" s="5">
-        <v>0.006</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="I7" s="4">
         <v>1</v>
@@ -700,10 +829,10 @@
         <v>2</v>
       </c>
       <c r="L7" s="4">
-        <v>0.059</v>
+        <v>5.8999999999999997E-2</v>
       </c>
       <c r="M7" s="5">
-        <v>0.047</v>
+        <v>4.7E-2</v>
       </c>
       <c r="N7" s="4">
         <v>1</v>
@@ -712,16 +841,16 @@
         <v>2</v>
       </c>
       <c r="Q7" s="5">
-        <v>0.051</v>
+        <v>5.0999999999999997E-2</v>
       </c>
       <c r="R7" s="5">
-        <v>0.004</v>
+        <v>4.0000000000000001E-3</v>
       </c>
       <c r="S7" s="4">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:19">
+    <row r="10" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
@@ -735,7 +864,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:19">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>6</v>
       </c>
@@ -749,7 +878,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:19">
+    <row r="12" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>5</v>
       </c>
@@ -763,7 +892,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:19">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
       <c r="B13" s="3" t="s">
         <v>0</v>
       </c>
@@ -801,7 +930,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:19">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>0</v>
       </c>
@@ -809,10 +938,10 @@
         <v>1</v>
       </c>
       <c r="C14" s="4">
-        <v>0.393</v>
+        <v>0.39300000000000002</v>
       </c>
       <c r="D14" s="4">
-        <v>0.056</v>
+        <v>5.6000000000000001E-2</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>0</v>
@@ -821,10 +950,10 @@
         <v>1</v>
       </c>
       <c r="H14" s="4">
-        <v>0.619</v>
+        <v>0.61899999999999999</v>
       </c>
       <c r="I14" s="5">
-        <v>0.024</v>
+        <v>2.4E-2</v>
       </c>
       <c r="K14" s="3" t="s">
         <v>0</v>
@@ -833,10 +962,10 @@
         <v>1</v>
       </c>
       <c r="M14" s="4">
-        <v>0.9429999999999999</v>
+        <v>0.94299999999999995</v>
       </c>
       <c r="N14" s="5">
-        <v>0.013</v>
+        <v>1.2999999999999999E-2</v>
       </c>
       <c r="P14" s="3" t="s">
         <v>0</v>
@@ -845,71 +974,71 @@
         <v>1</v>
       </c>
       <c r="R14" s="4">
-        <v>0.228</v>
+        <v>0.22800000000000001</v>
       </c>
       <c r="S14" s="4">
         <v>0.06</v>
       </c>
     </row>
-    <row r="15" spans="1:19">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B15" s="4">
-        <v>0.393</v>
+        <v>0.39300000000000002</v>
       </c>
       <c r="C15" s="4">
         <v>1</v>
       </c>
       <c r="D15" s="4">
-        <v>0.202</v>
+        <v>0.20200000000000001</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>1</v>
       </c>
       <c r="G15" s="4">
-        <v>0.619</v>
+        <v>0.61899999999999999</v>
       </c>
       <c r="H15" s="4">
         <v>1</v>
       </c>
       <c r="I15" s="5">
-        <v>0.011</v>
+        <v>1.0999999999999999E-2</v>
       </c>
       <c r="K15" s="3" t="s">
         <v>1</v>
       </c>
       <c r="L15" s="4">
-        <v>0.9429999999999999</v>
+        <v>0.94299999999999995</v>
       </c>
       <c r="M15" s="4">
         <v>1</v>
       </c>
       <c r="N15" s="5">
-        <v>0.013</v>
+        <v>1.2999999999999999E-2</v>
       </c>
       <c r="P15" s="3" t="s">
         <v>1</v>
       </c>
       <c r="Q15" s="4">
-        <v>0.228</v>
+        <v>0.22800000000000001</v>
       </c>
       <c r="R15" s="4">
         <v>1</v>
       </c>
       <c r="S15" s="5">
-        <v>0.003</v>
-      </c>
-    </row>
-    <row r="16" spans="1:19">
+        <v>3.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B16" s="4">
-        <v>0.056</v>
+        <v>5.6000000000000001E-2</v>
       </c>
       <c r="C16" s="4">
-        <v>0.202</v>
+        <v>0.20200000000000001</v>
       </c>
       <c r="D16" s="4">
         <v>1</v>
@@ -918,10 +1047,10 @@
         <v>2</v>
       </c>
       <c r="G16" s="5">
-        <v>0.024</v>
+        <v>2.4E-2</v>
       </c>
       <c r="H16" s="5">
-        <v>0.011</v>
+        <v>1.0999999999999999E-2</v>
       </c>
       <c r="I16" s="4">
         <v>1</v>
@@ -930,10 +1059,10 @@
         <v>2</v>
       </c>
       <c r="L16" s="5">
-        <v>0.013</v>
+        <v>1.2999999999999999E-2</v>
       </c>
       <c r="M16" s="5">
-        <v>0.013</v>
+        <v>1.2999999999999999E-2</v>
       </c>
       <c r="N16" s="4">
         <v>1</v>
@@ -945,55 +1074,127 @@
         <v>0.06</v>
       </c>
       <c r="R16" s="5">
-        <v>0.003</v>
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="S16" s="4">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:19">
-      <c r="A19" s="1" t="s">
+    <row r="17" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A18" s="6"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="7"/>
+      <c r="J18" s="7"/>
+      <c r="K18" s="7"/>
+      <c r="L18" s="7"/>
+      <c r="M18" s="7"/>
+      <c r="N18" s="7"/>
+      <c r="O18" s="7"/>
+      <c r="P18" s="7"/>
+      <c r="Q18" s="7"/>
+      <c r="R18" s="7"/>
+      <c r="S18" s="7"/>
+      <c r="T18" s="8"/>
+    </row>
+    <row r="19" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="K19" s="1" t="s">
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="P19" s="1" t="s">
+      <c r="L19" s="10"/>
+      <c r="M19" s="10"/>
+      <c r="N19" s="10"/>
+      <c r="O19" s="10"/>
+      <c r="P19" s="11" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="20" spans="1:19">
-      <c r="A20" s="2" t="s">
+      <c r="Q19" s="10"/>
+      <c r="R19" s="10"/>
+      <c r="S19" s="10"/>
+      <c r="T19" s="12"/>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A20" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="F20" s="2" t="s">
+      <c r="B20" s="10"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="K20" s="2" t="s">
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="10"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="P20" s="2" t="s">
+      <c r="L20" s="10"/>
+      <c r="M20" s="10"/>
+      <c r="N20" s="10"/>
+      <c r="O20" s="10"/>
+      <c r="P20" s="14" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="21" spans="1:19">
-      <c r="A21" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="K21" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="P21" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="22" spans="1:19">
+      <c r="Q20" s="10"/>
+      <c r="R20" s="10"/>
+      <c r="S20" s="10"/>
+      <c r="T20" s="12"/>
+    </row>
+    <row r="21" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A21" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="G21" s="10"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="10"/>
+      <c r="J21" s="10"/>
+      <c r="K21" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="L21" s="10"/>
+      <c r="M21" s="10"/>
+      <c r="N21" s="10"/>
+      <c r="O21" s="10"/>
+      <c r="P21" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q21" s="10"/>
+      <c r="R21" s="10"/>
+      <c r="S21" s="10"/>
+      <c r="T21" s="12"/>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A22" s="15"/>
       <c r="B22" s="3" t="s">
         <v>0</v>
       </c>
@@ -1003,6 +1204,8 @@
       <c r="D22" s="3" t="s">
         <v>2</v>
       </c>
+      <c r="E22" s="10"/>
+      <c r="F22" s="10"/>
       <c r="G22" s="3" t="s">
         <v>0</v>
       </c>
@@ -1012,6 +1215,8 @@
       <c r="I22" s="3" t="s">
         <v>2</v>
       </c>
+      <c r="J22" s="10"/>
+      <c r="K22" s="10"/>
       <c r="L22" s="3" t="s">
         <v>0</v>
       </c>
@@ -1021,6 +1226,8 @@
       <c r="N22" s="3" t="s">
         <v>2</v>
       </c>
+      <c r="O22" s="10"/>
+      <c r="P22" s="10"/>
       <c r="Q22" s="3" t="s">
         <v>0</v>
       </c>
@@ -1030,200 +1237,306 @@
       <c r="S22" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="23" spans="1:19">
-      <c r="A23" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B23" s="4">
-        <v>1</v>
-      </c>
-      <c r="C23" s="4">
-        <v>0.831</v>
-      </c>
-      <c r="D23" s="5">
-        <v>0.016</v>
-      </c>
+      <c r="T22" s="12"/>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A23" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="B23" s="17">
+        <v>1</v>
+      </c>
+      <c r="C23" s="17">
+        <v>0.83099999999999996</v>
+      </c>
+      <c r="D23" s="18">
+        <v>1.6E-2</v>
+      </c>
+      <c r="E23" s="10"/>
       <c r="F23" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="G23" s="4">
-        <v>1</v>
-      </c>
-      <c r="H23" s="4">
-        <v>0.321</v>
-      </c>
-      <c r="I23" s="5">
-        <v>0.005</v>
-      </c>
+      <c r="G23" s="17">
+        <v>1</v>
+      </c>
+      <c r="H23" s="17">
+        <v>0.32100000000000001</v>
+      </c>
+      <c r="I23" s="18">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J23" s="10"/>
       <c r="K23" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="L23" s="4">
-        <v>1</v>
-      </c>
-      <c r="M23" s="4">
-        <v>0.394</v>
-      </c>
-      <c r="N23" s="5">
-        <v>0.038</v>
-      </c>
+      <c r="L23" s="17">
+        <v>1</v>
+      </c>
+      <c r="M23" s="17">
+        <v>0.39400000000000002</v>
+      </c>
+      <c r="N23" s="18">
+        <v>3.7999999999999999E-2</v>
+      </c>
+      <c r="O23" s="10"/>
       <c r="P23" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="Q23" s="4">
-        <v>1</v>
-      </c>
-      <c r="R23" s="4">
-        <v>0.288</v>
-      </c>
-      <c r="S23" s="5">
-        <v>0.004</v>
-      </c>
-    </row>
-    <row r="24" spans="1:19">
-      <c r="A24" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B24" s="4">
-        <v>0.831</v>
-      </c>
-      <c r="C24" s="4">
-        <v>1</v>
-      </c>
-      <c r="D24" s="5">
-        <v>0.016</v>
-      </c>
+      <c r="Q23" s="17">
+        <v>1</v>
+      </c>
+      <c r="R23" s="17">
+        <v>0.28799999999999998</v>
+      </c>
+      <c r="S23" s="18">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="T23" s="12"/>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A24" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="B24" s="17">
+        <v>0.83099999999999996</v>
+      </c>
+      <c r="C24" s="17">
+        <v>1</v>
+      </c>
+      <c r="D24" s="18">
+        <v>1.6E-2</v>
+      </c>
+      <c r="E24" s="10"/>
       <c r="F24" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="G24" s="4">
-        <v>0.321</v>
-      </c>
-      <c r="H24" s="4">
-        <v>1</v>
-      </c>
-      <c r="I24" s="5">
-        <v>0.046</v>
-      </c>
+      <c r="G24" s="17">
+        <v>0.32100000000000001</v>
+      </c>
+      <c r="H24" s="17">
+        <v>1</v>
+      </c>
+      <c r="I24" s="18">
+        <v>4.5999999999999999E-2</v>
+      </c>
+      <c r="J24" s="10"/>
       <c r="K24" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="L24" s="4">
-        <v>0.394</v>
-      </c>
-      <c r="M24" s="4">
-        <v>1</v>
-      </c>
-      <c r="N24" s="5">
-        <v>0.006</v>
-      </c>
+      <c r="L24" s="17">
+        <v>0.39400000000000002</v>
+      </c>
+      <c r="M24" s="17">
+        <v>1</v>
+      </c>
+      <c r="N24" s="18">
+        <v>6.0000000000000001E-3</v>
+      </c>
+      <c r="O24" s="10"/>
       <c r="P24" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="Q24" s="4">
-        <v>0.288</v>
-      </c>
-      <c r="R24" s="4">
-        <v>1</v>
-      </c>
-      <c r="S24" s="5">
+      <c r="Q24" s="17">
+        <v>0.28799999999999998</v>
+      </c>
+      <c r="R24" s="17">
+        <v>1</v>
+      </c>
+      <c r="S24" s="18">
         <v>0.05</v>
       </c>
-    </row>
-    <row r="25" spans="1:19">
-      <c r="A25" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B25" s="5">
-        <v>0.016</v>
-      </c>
-      <c r="C25" s="5">
-        <v>0.016</v>
-      </c>
-      <c r="D25" s="4">
-        <v>1</v>
-      </c>
+      <c r="T24" s="12"/>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A25" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="B25" s="18">
+        <v>1.6E-2</v>
+      </c>
+      <c r="C25" s="18">
+        <v>1.6E-2</v>
+      </c>
+      <c r="D25" s="17">
+        <v>1</v>
+      </c>
+      <c r="E25" s="10"/>
       <c r="F25" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="G25" s="5">
-        <v>0.005</v>
-      </c>
-      <c r="H25" s="5">
-        <v>0.046</v>
-      </c>
-      <c r="I25" s="4">
-        <v>1</v>
-      </c>
+      <c r="G25" s="18">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="H25" s="18">
+        <v>4.5999999999999999E-2</v>
+      </c>
+      <c r="I25" s="17">
+        <v>1</v>
+      </c>
+      <c r="J25" s="10"/>
       <c r="K25" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="L25" s="5">
-        <v>0.038</v>
-      </c>
-      <c r="M25" s="5">
-        <v>0.006</v>
-      </c>
-      <c r="N25" s="4">
-        <v>1</v>
-      </c>
+      <c r="L25" s="18">
+        <v>3.7999999999999999E-2</v>
+      </c>
+      <c r="M25" s="18">
+        <v>6.0000000000000001E-3</v>
+      </c>
+      <c r="N25" s="17">
+        <v>1</v>
+      </c>
+      <c r="O25" s="10"/>
       <c r="P25" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="Q25" s="5">
-        <v>0.004</v>
-      </c>
-      <c r="R25" s="5">
+      <c r="Q25" s="18">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="R25" s="18">
         <v>0.05</v>
       </c>
-      <c r="S25" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:19">
-      <c r="A28" s="1" t="s">
+      <c r="S25" s="17">
+        <v>1</v>
+      </c>
+      <c r="T25" s="12"/>
+    </row>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A26" s="15"/>
+      <c r="B26" s="10"/>
+      <c r="C26" s="10"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="10"/>
+      <c r="H26" s="10"/>
+      <c r="I26" s="10"/>
+      <c r="J26" s="10"/>
+      <c r="K26" s="10"/>
+      <c r="L26" s="10"/>
+      <c r="M26" s="10"/>
+      <c r="N26" s="10"/>
+      <c r="O26" s="10"/>
+      <c r="P26" s="10"/>
+      <c r="Q26" s="10"/>
+      <c r="R26" s="10"/>
+      <c r="S26" s="10"/>
+      <c r="T26" s="12"/>
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A27" s="15"/>
+      <c r="B27" s="10"/>
+      <c r="C27" s="10"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="10"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="10"/>
+      <c r="H27" s="10"/>
+      <c r="I27" s="10"/>
+      <c r="J27" s="10"/>
+      <c r="K27" s="10"/>
+      <c r="L27" s="10"/>
+      <c r="M27" s="10"/>
+      <c r="N27" s="10"/>
+      <c r="O27" s="10"/>
+      <c r="P27" s="10"/>
+      <c r="Q27" s="10"/>
+      <c r="R27" s="10"/>
+      <c r="S27" s="10"/>
+      <c r="T27" s="12"/>
+    </row>
+    <row r="28" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A28" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="B28" s="10"/>
+      <c r="C28" s="10"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="10"/>
+      <c r="F28" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="K28" s="1" t="s">
+      <c r="G28" s="10"/>
+      <c r="H28" s="10"/>
+      <c r="I28" s="10"/>
+      <c r="J28" s="10"/>
+      <c r="K28" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="P28" s="1" t="s">
+      <c r="L28" s="10"/>
+      <c r="M28" s="10"/>
+      <c r="N28" s="10"/>
+      <c r="O28" s="10"/>
+      <c r="P28" s="11" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="29" spans="1:19">
-      <c r="A29" s="2" t="s">
+      <c r="Q28" s="10"/>
+      <c r="R28" s="10"/>
+      <c r="S28" s="10"/>
+      <c r="T28" s="12"/>
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A29" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="F29" s="2" t="s">
+      <c r="B29" s="10"/>
+      <c r="C29" s="10"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="K29" s="2" t="s">
+      <c r="G29" s="10"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="P29" s="2" t="s">
+      <c r="L29" s="10"/>
+      <c r="M29" s="10"/>
+      <c r="N29" s="10"/>
+      <c r="O29" s="10"/>
+      <c r="P29" s="14" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="30" spans="1:19">
-      <c r="A30" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="K30" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="P30" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="31" spans="1:19">
+      <c r="Q29" s="10"/>
+      <c r="R29" s="10"/>
+      <c r="S29" s="10"/>
+      <c r="T29" s="12"/>
+    </row>
+    <row r="30" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A30" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B30" s="10"/>
+      <c r="C30" s="10"/>
+      <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="G30" s="10"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="10"/>
+      <c r="J30" s="10"/>
+      <c r="K30" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="L30" s="10"/>
+      <c r="M30" s="10"/>
+      <c r="N30" s="10"/>
+      <c r="O30" s="10"/>
+      <c r="P30" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q30" s="10"/>
+      <c r="R30" s="10"/>
+      <c r="S30" s="10"/>
+      <c r="T30" s="12"/>
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A31" s="15"/>
       <c r="B31" s="3" t="s">
         <v>0</v>
       </c>
@@ -1233,6 +1546,8 @@
       <c r="D31" s="3" t="s">
         <v>2</v>
       </c>
+      <c r="E31" s="10"/>
+      <c r="F31" s="10"/>
       <c r="G31" s="3" t="s">
         <v>0</v>
       </c>
@@ -1242,6 +1557,8 @@
       <c r="I31" s="3" t="s">
         <v>2</v>
       </c>
+      <c r="J31" s="10"/>
+      <c r="K31" s="10"/>
       <c r="L31" s="3" t="s">
         <v>0</v>
       </c>
@@ -1251,6 +1568,8 @@
       <c r="N31" s="3" t="s">
         <v>2</v>
       </c>
+      <c r="O31" s="10"/>
+      <c r="P31" s="10"/>
       <c r="Q31" s="3" t="s">
         <v>0</v>
       </c>
@@ -1260,158 +1579,193 @@
       <c r="S31" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="32" spans="1:19">
-      <c r="A32" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B32" s="4">
-        <v>1</v>
-      </c>
-      <c r="C32" s="4">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="D32" s="4">
-        <v>0.6899999999999999</v>
-      </c>
+      <c r="T31" s="12"/>
+    </row>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A32" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="B32" s="17">
+        <v>1</v>
+      </c>
+      <c r="C32" s="17">
+        <v>0.69</v>
+      </c>
+      <c r="D32" s="17">
+        <v>0.69</v>
+      </c>
+      <c r="E32" s="10"/>
       <c r="F32" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="G32" s="4">
-        <v>1</v>
-      </c>
-      <c r="H32" s="4">
+      <c r="G32" s="17">
+        <v>1</v>
+      </c>
+      <c r="H32" s="17">
         <v>0.436</v>
       </c>
-      <c r="I32" s="5">
-        <v>0.007</v>
-      </c>
+      <c r="I32" s="18">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="J32" s="10"/>
       <c r="K32" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="L32" s="4">
-        <v>1</v>
-      </c>
-      <c r="M32" s="4">
-        <v>0.523</v>
-      </c>
-      <c r="N32" s="5">
-        <v>0.029</v>
-      </c>
+      <c r="L32" s="17">
+        <v>1</v>
+      </c>
+      <c r="M32" s="17">
+        <v>0.52300000000000002</v>
+      </c>
+      <c r="N32" s="18">
+        <v>2.9000000000000001E-2</v>
+      </c>
+      <c r="O32" s="10"/>
       <c r="P32" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="Q32" s="4">
-        <v>1</v>
-      </c>
-      <c r="R32" s="4">
-        <v>0.57</v>
-      </c>
-      <c r="S32" s="5">
+      <c r="Q32" s="17">
+        <v>1</v>
+      </c>
+      <c r="R32" s="17">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="S32" s="18">
         <v>0.01</v>
       </c>
-    </row>
-    <row r="33" spans="1:19">
-      <c r="A33" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B33" s="4">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="C33" s="4">
-        <v>1</v>
-      </c>
-      <c r="D33" s="4">
-        <v>0.6899999999999999</v>
-      </c>
+      <c r="T32" s="12"/>
+    </row>
+    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A33" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="B33" s="17">
+        <v>0.69</v>
+      </c>
+      <c r="C33" s="17">
+        <v>1</v>
+      </c>
+      <c r="D33" s="17">
+        <v>0.69</v>
+      </c>
+      <c r="E33" s="10"/>
       <c r="F33" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="G33" s="4">
+      <c r="G33" s="17">
         <v>0.436</v>
       </c>
-      <c r="H33" s="4">
-        <v>1</v>
-      </c>
-      <c r="I33" s="5">
-        <v>0.035</v>
-      </c>
+      <c r="H33" s="17">
+        <v>1</v>
+      </c>
+      <c r="I33" s="18">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="J33" s="10"/>
       <c r="K33" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="L33" s="4">
-        <v>0.523</v>
-      </c>
-      <c r="M33" s="4">
-        <v>1</v>
-      </c>
-      <c r="N33" s="5">
-        <v>0.008999999999999999</v>
-      </c>
+      <c r="L33" s="17">
+        <v>0.52300000000000002</v>
+      </c>
+      <c r="M33" s="17">
+        <v>1</v>
+      </c>
+      <c r="N33" s="18">
+        <v>8.9999999999999993E-3</v>
+      </c>
+      <c r="O33" s="10"/>
       <c r="P33" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="Q33" s="4">
-        <v>0.57</v>
-      </c>
-      <c r="R33" s="4">
-        <v>1</v>
-      </c>
-      <c r="S33" s="5">
-        <v>0.026</v>
-      </c>
-    </row>
-    <row r="34" spans="1:19">
-      <c r="A34" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B34" s="4">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="C34" s="4">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="D34" s="4">
-        <v>1</v>
-      </c>
+      <c r="Q33" s="17">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="R33" s="17">
+        <v>1</v>
+      </c>
+      <c r="S33" s="18">
+        <v>2.5999999999999999E-2</v>
+      </c>
+      <c r="T33" s="12"/>
+    </row>
+    <row r="34" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A34" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="B34" s="17">
+        <v>0.69</v>
+      </c>
+      <c r="C34" s="17">
+        <v>0.69</v>
+      </c>
+      <c r="D34" s="17">
+        <v>1</v>
+      </c>
+      <c r="E34" s="10"/>
       <c r="F34" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="G34" s="5">
-        <v>0.007</v>
-      </c>
-      <c r="H34" s="5">
-        <v>0.035</v>
-      </c>
-      <c r="I34" s="4">
-        <v>1</v>
-      </c>
+      <c r="G34" s="18">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="H34" s="18">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="I34" s="17">
+        <v>1</v>
+      </c>
+      <c r="J34" s="10"/>
       <c r="K34" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="L34" s="5">
-        <v>0.029</v>
-      </c>
-      <c r="M34" s="5">
-        <v>0.008999999999999999</v>
-      </c>
-      <c r="N34" s="4">
-        <v>1</v>
-      </c>
+      <c r="L34" s="18">
+        <v>2.9000000000000001E-2</v>
+      </c>
+      <c r="M34" s="18">
+        <v>8.9999999999999993E-3</v>
+      </c>
+      <c r="N34" s="17">
+        <v>1</v>
+      </c>
+      <c r="O34" s="10"/>
       <c r="P34" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="Q34" s="5">
+      <c r="Q34" s="18">
         <v>0.01</v>
       </c>
-      <c r="R34" s="5">
-        <v>0.026</v>
-      </c>
-      <c r="S34" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:19">
+      <c r="R34" s="18">
+        <v>2.5999999999999999E-2</v>
+      </c>
+      <c r="S34" s="17">
+        <v>1</v>
+      </c>
+      <c r="T34" s="12"/>
+    </row>
+    <row r="35" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="19"/>
+      <c r="B35" s="20"/>
+      <c r="C35" s="20"/>
+      <c r="D35" s="20"/>
+      <c r="E35" s="20"/>
+      <c r="F35" s="20"/>
+      <c r="G35" s="20"/>
+      <c r="H35" s="20"/>
+      <c r="I35" s="20"/>
+      <c r="J35" s="20"/>
+      <c r="K35" s="20"/>
+      <c r="L35" s="20"/>
+      <c r="M35" s="20"/>
+      <c r="N35" s="20"/>
+      <c r="O35" s="20"/>
+      <c r="P35" s="20"/>
+      <c r="Q35" s="20"/>
+      <c r="R35" s="20"/>
+      <c r="S35" s="20"/>
+      <c r="T35" s="21"/>
+    </row>
+    <row r="37" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>3</v>
       </c>
@@ -1425,7 +1779,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="38" spans="1:19">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>9</v>
       </c>
@@ -1439,7 +1793,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="39" spans="1:19">
+    <row r="39" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>5</v>
       </c>
@@ -1453,7 +1807,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:19">
+    <row r="40" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B40" s="3" t="s">
         <v>0</v>
       </c>
@@ -1491,7 +1845,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="1:19">
+    <row r="41" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
         <v>0</v>
       </c>
@@ -1499,10 +1853,10 @@
         <v>1</v>
       </c>
       <c r="C41" s="4">
-        <v>0.492</v>
+        <v>0.49199999999999999</v>
       </c>
       <c r="D41" s="4">
-        <v>0.467</v>
+        <v>0.46700000000000003</v>
       </c>
       <c r="F41" s="3" t="s">
         <v>0</v>
@@ -1514,7 +1868,7 @@
         <v>0.318</v>
       </c>
       <c r="I41" s="5">
-        <v>0.004</v>
+        <v>4.0000000000000001E-3</v>
       </c>
       <c r="K41" s="3" t="s">
         <v>0</v>
@@ -1523,10 +1877,10 @@
         <v>1</v>
       </c>
       <c r="M41" s="4">
-        <v>0.321</v>
+        <v>0.32100000000000001</v>
       </c>
       <c r="N41" s="5">
-        <v>0.005</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="P41" s="3" t="s">
         <v>0</v>
@@ -1535,24 +1889,24 @@
         <v>1</v>
       </c>
       <c r="R41" s="4">
-        <v>0.089</v>
+        <v>8.8999999999999996E-2</v>
       </c>
       <c r="S41" s="4">
-        <v>0.089</v>
-      </c>
-    </row>
-    <row r="42" spans="1:19">
+        <v>8.8999999999999996E-2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A42" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B42" s="4">
-        <v>0.492</v>
+        <v>0.49199999999999999</v>
       </c>
       <c r="C42" s="4">
         <v>1</v>
       </c>
       <c r="D42" s="4">
-        <v>0.267</v>
+        <v>0.26700000000000002</v>
       </c>
       <c r="F42" s="3" t="s">
         <v>1</v>
@@ -1564,42 +1918,42 @@
         <v>1</v>
       </c>
       <c r="I42" s="5">
-        <v>0.044</v>
+        <v>4.3999999999999997E-2</v>
       </c>
       <c r="K42" s="3" t="s">
         <v>1</v>
       </c>
       <c r="L42" s="4">
-        <v>0.321</v>
+        <v>0.32100000000000001</v>
       </c>
       <c r="M42" s="4">
         <v>1</v>
       </c>
       <c r="N42" s="5">
-        <v>0.046</v>
+        <v>4.5999999999999999E-2</v>
       </c>
       <c r="P42" s="3" t="s">
         <v>1</v>
       </c>
       <c r="Q42" s="4">
-        <v>0.089</v>
+        <v>8.8999999999999996E-2</v>
       </c>
       <c r="R42" s="4">
         <v>1</v>
       </c>
       <c r="S42" s="5">
-        <v>0.001</v>
-      </c>
-    </row>
-    <row r="43" spans="1:19">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B43" s="4">
-        <v>0.467</v>
+        <v>0.46700000000000003</v>
       </c>
       <c r="C43" s="4">
-        <v>0.267</v>
+        <v>0.26700000000000002</v>
       </c>
       <c r="D43" s="4">
         <v>1</v>
@@ -1608,10 +1962,10 @@
         <v>2</v>
       </c>
       <c r="G43" s="5">
-        <v>0.004</v>
+        <v>4.0000000000000001E-3</v>
       </c>
       <c r="H43" s="5">
-        <v>0.044</v>
+        <v>4.3999999999999997E-2</v>
       </c>
       <c r="I43" s="4">
         <v>1</v>
@@ -1620,10 +1974,10 @@
         <v>2</v>
       </c>
       <c r="L43" s="5">
-        <v>0.005</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="M43" s="5">
-        <v>0.046</v>
+        <v>4.5999999999999999E-2</v>
       </c>
       <c r="N43" s="4">
         <v>1</v>
@@ -1632,16 +1986,16 @@
         <v>2</v>
       </c>
       <c r="Q43" s="4">
-        <v>0.089</v>
+        <v>8.8999999999999996E-2</v>
       </c>
       <c r="R43" s="5">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="S43" s="4">
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:19">
+    <row r="46" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>3</v>
       </c>
@@ -1655,7 +2009,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="47" spans="1:19">
+    <row r="47" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>10</v>
       </c>
@@ -1669,7 +2023,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="48" spans="1:19">
+    <row r="48" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>5</v>
       </c>
@@ -1683,7 +2037,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="49" spans="1:19">
+    <row r="49" spans="1:19" x14ac:dyDescent="0.3">
       <c r="B49" s="3" t="s">
         <v>0</v>
       </c>
@@ -1721,7 +2075,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="50" spans="1:19">
+    <row r="50" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A50" s="3" t="s">
         <v>0</v>
       </c>
@@ -1729,10 +2083,10 @@
         <v>1</v>
       </c>
       <c r="C50" s="4">
-        <v>0.305</v>
+        <v>0.30499999999999999</v>
       </c>
       <c r="D50" s="4">
-        <v>0.453</v>
+        <v>0.45300000000000001</v>
       </c>
       <c r="F50" s="3" t="s">
         <v>0</v>
@@ -1741,10 +2095,10 @@
         <v>1</v>
       </c>
       <c r="H50" s="5">
-        <v>0.002</v>
+        <v>2E-3</v>
       </c>
       <c r="I50" s="4">
-        <v>0.083</v>
+        <v>8.3000000000000004E-2</v>
       </c>
       <c r="K50" s="3" t="s">
         <v>0</v>
@@ -1753,10 +2107,10 @@
         <v>1</v>
       </c>
       <c r="M50" s="5">
-        <v>0.024</v>
+        <v>2.4E-2</v>
       </c>
       <c r="N50" s="5">
-        <v>0.024</v>
+        <v>2.4E-2</v>
       </c>
       <c r="P50" s="3" t="s">
         <v>0</v>
@@ -1765,71 +2119,71 @@
         <v>1</v>
       </c>
       <c r="R50" s="5">
-        <v>0.018</v>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="S50" s="4">
-        <v>0.944</v>
-      </c>
-    </row>
-    <row r="51" spans="1:19">
+        <v>0.94399999999999995</v>
+      </c>
+    </row>
+    <row r="51" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B51" s="4">
-        <v>0.305</v>
+        <v>0.30499999999999999</v>
       </c>
       <c r="C51" s="4">
         <v>1</v>
       </c>
       <c r="D51" s="4">
-        <v>0.545</v>
+        <v>0.54500000000000004</v>
       </c>
       <c r="F51" s="3" t="s">
         <v>1</v>
       </c>
       <c r="G51" s="5">
-        <v>0.002</v>
+        <v>2E-3</v>
       </c>
       <c r="H51" s="4">
         <v>1</v>
       </c>
       <c r="I51" s="4">
-        <v>0.136</v>
+        <v>0.13600000000000001</v>
       </c>
       <c r="K51" s="3" t="s">
         <v>1</v>
       </c>
       <c r="L51" s="5">
-        <v>0.024</v>
+        <v>2.4E-2</v>
       </c>
       <c r="M51" s="4">
         <v>1</v>
       </c>
       <c r="N51" s="4">
-        <v>0.944</v>
+        <v>0.94399999999999995</v>
       </c>
       <c r="P51" s="3" t="s">
         <v>1</v>
       </c>
       <c r="Q51" s="5">
-        <v>0.018</v>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="R51" s="4">
         <v>1</v>
       </c>
       <c r="S51" s="5">
-        <v>0.018</v>
-      </c>
-    </row>
-    <row r="52" spans="1:19">
+        <v>1.7999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A52" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B52" s="4">
-        <v>0.453</v>
+        <v>0.45300000000000001</v>
       </c>
       <c r="C52" s="4">
-        <v>0.545</v>
+        <v>0.54500000000000004</v>
       </c>
       <c r="D52" s="4">
         <v>1</v>
@@ -1838,10 +2192,10 @@
         <v>2</v>
       </c>
       <c r="G52" s="4">
-        <v>0.083</v>
+        <v>8.3000000000000004E-2</v>
       </c>
       <c r="H52" s="4">
-        <v>0.136</v>
+        <v>0.13600000000000001</v>
       </c>
       <c r="I52" s="4">
         <v>1</v>
@@ -1850,10 +2204,10 @@
         <v>2</v>
       </c>
       <c r="L52" s="5">
-        <v>0.024</v>
+        <v>2.4E-2</v>
       </c>
       <c r="M52" s="4">
-        <v>0.944</v>
+        <v>0.94399999999999995</v>
       </c>
       <c r="N52" s="4">
         <v>1</v>
@@ -1862,10 +2216,10 @@
         <v>2</v>
       </c>
       <c r="Q52" s="4">
-        <v>0.944</v>
+        <v>0.94399999999999995</v>
       </c>
       <c r="R52" s="5">
-        <v>0.018</v>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="S52" s="4">
         <v>1</v>

</xml_diff>

<commit_message>
several changes in paper and median data added
</commit_message>
<xml_diff>
--- a/Data/KW_dunn_between_month.xlsx
+++ b/Data/KW_dunn_between_month.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yaroslav\OneDrive\Рабочий стол\Python_repos\Python_projects_ICG_SB_RAS\Four_host_species_OF\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF730FCA-C22C-4E4E-96DD-0DE1519966D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B084CE1A-782E-4B79-AB86-D01107B6925C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="KW_dunn_between_month" sheetId="1" r:id="rId1"/>
@@ -286,7 +286,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -299,17 +299,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -1107,94 +1102,49 @@
       <c r="A19" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B19" s="10"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="11" t="s">
+      <c r="F19" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G19" s="10"/>
-      <c r="H19" s="10"/>
-      <c r="I19" s="10"/>
-      <c r="J19" s="10"/>
-      <c r="K19" s="11" t="s">
+      <c r="K19" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="L19" s="10"/>
-      <c r="M19" s="10"/>
-      <c r="N19" s="10"/>
-      <c r="O19" s="10"/>
-      <c r="P19" s="11" t="s">
+      <c r="P19" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Q19" s="10"/>
-      <c r="R19" s="10"/>
-      <c r="S19" s="10"/>
-      <c r="T19" s="12"/>
+      <c r="T19" s="10"/>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A20" s="13" t="s">
+      <c r="A20" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="14" t="s">
+      <c r="F20" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G20" s="10"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="10"/>
-      <c r="J20" s="10"/>
-      <c r="K20" s="14" t="s">
+      <c r="K20" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="L20" s="10"/>
-      <c r="M20" s="10"/>
-      <c r="N20" s="10"/>
-      <c r="O20" s="10"/>
-      <c r="P20" s="14" t="s">
+      <c r="P20" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="Q20" s="10"/>
-      <c r="R20" s="10"/>
-      <c r="S20" s="10"/>
-      <c r="T20" s="12"/>
+      <c r="T20" s="10"/>
     </row>
     <row r="21" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="B21" s="10"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="G21" s="10"/>
-      <c r="H21" s="10"/>
-      <c r="I21" s="10"/>
-      <c r="J21" s="10"/>
-      <c r="K21" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="L21" s="10"/>
-      <c r="M21" s="10"/>
-      <c r="N21" s="10"/>
-      <c r="O21" s="10"/>
-      <c r="P21" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="Q21" s="10"/>
-      <c r="R21" s="10"/>
-      <c r="S21" s="10"/>
-      <c r="T21" s="12"/>
+      <c r="F21" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="P21" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="T21" s="10"/>
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A22" s="15"/>
+      <c r="A22" s="12"/>
       <c r="B22" s="3" t="s">
         <v>0</v>
       </c>
@@ -1204,8 +1154,6 @@
       <c r="D22" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
       <c r="G22" s="3" t="s">
         <v>0</v>
       </c>
@@ -1215,8 +1163,6 @@
       <c r="I22" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="J22" s="10"/>
-      <c r="K22" s="10"/>
       <c r="L22" s="3" t="s">
         <v>0</v>
       </c>
@@ -1226,8 +1172,6 @@
       <c r="N22" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="O22" s="10"/>
-      <c r="P22" s="10"/>
       <c r="Q22" s="3" t="s">
         <v>0</v>
       </c>
@@ -1237,306 +1181,216 @@
       <c r="S22" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="T22" s="12"/>
+      <c r="T22" s="10"/>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A23" s="16" t="s">
-        <v>0</v>
-      </c>
-      <c r="B23" s="17">
-        <v>1</v>
-      </c>
-      <c r="C23" s="17">
+      <c r="A23" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B23" s="4">
+        <v>1</v>
+      </c>
+      <c r="C23" s="4">
         <v>0.83099999999999996</v>
       </c>
-      <c r="D23" s="18">
+      <c r="D23" s="5">
         <v>1.6E-2</v>
       </c>
-      <c r="E23" s="10"/>
       <c r="F23" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="G23" s="17">
-        <v>1</v>
-      </c>
-      <c r="H23" s="17">
+      <c r="G23" s="4">
+        <v>1</v>
+      </c>
+      <c r="H23" s="4">
         <v>0.32100000000000001</v>
       </c>
-      <c r="I23" s="18">
+      <c r="I23" s="5">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="J23" s="10"/>
       <c r="K23" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="L23" s="17">
-        <v>1</v>
-      </c>
-      <c r="M23" s="17">
+      <c r="L23" s="4">
+        <v>1</v>
+      </c>
+      <c r="M23" s="4">
         <v>0.39400000000000002</v>
       </c>
-      <c r="N23" s="18">
+      <c r="N23" s="5">
         <v>3.7999999999999999E-2</v>
       </c>
-      <c r="O23" s="10"/>
       <c r="P23" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="Q23" s="17">
-        <v>1</v>
-      </c>
-      <c r="R23" s="17">
+      <c r="Q23" s="4">
+        <v>1</v>
+      </c>
+      <c r="R23" s="4">
         <v>0.28799999999999998</v>
       </c>
-      <c r="S23" s="18">
+      <c r="S23" s="5">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="T23" s="12"/>
+      <c r="T23" s="10"/>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A24" s="16" t="s">
-        <v>1</v>
-      </c>
-      <c r="B24" s="17">
+      <c r="A24" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="B24" s="4">
         <v>0.83099999999999996</v>
       </c>
-      <c r="C24" s="17">
-        <v>1</v>
-      </c>
-      <c r="D24" s="18">
+      <c r="C24" s="4">
+        <v>1</v>
+      </c>
+      <c r="D24" s="5">
         <v>1.6E-2</v>
       </c>
-      <c r="E24" s="10"/>
       <c r="F24" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="G24" s="17">
+      <c r="G24" s="4">
         <v>0.32100000000000001</v>
       </c>
-      <c r="H24" s="17">
-        <v>1</v>
-      </c>
-      <c r="I24" s="18">
+      <c r="H24" s="4">
+        <v>1</v>
+      </c>
+      <c r="I24" s="5">
         <v>4.5999999999999999E-2</v>
       </c>
-      <c r="J24" s="10"/>
       <c r="K24" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="L24" s="17">
+      <c r="L24" s="4">
         <v>0.39400000000000002</v>
       </c>
-      <c r="M24" s="17">
-        <v>1</v>
-      </c>
-      <c r="N24" s="18">
+      <c r="M24" s="4">
+        <v>1</v>
+      </c>
+      <c r="N24" s="5">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="O24" s="10"/>
       <c r="P24" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="Q24" s="17">
+      <c r="Q24" s="4">
         <v>0.28799999999999998</v>
       </c>
-      <c r="R24" s="17">
-        <v>1</v>
-      </c>
-      <c r="S24" s="18">
+      <c r="R24" s="4">
+        <v>1</v>
+      </c>
+      <c r="S24" s="5">
         <v>0.05</v>
       </c>
-      <c r="T24" s="12"/>
+      <c r="T24" s="10"/>
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A25" s="16" t="s">
-        <v>2</v>
-      </c>
-      <c r="B25" s="18">
+      <c r="A25" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B25" s="5">
         <v>1.6E-2</v>
       </c>
-      <c r="C25" s="18">
+      <c r="C25" s="5">
         <v>1.6E-2</v>
       </c>
-      <c r="D25" s="17">
-        <v>1</v>
-      </c>
-      <c r="E25" s="10"/>
+      <c r="D25" s="4">
+        <v>1</v>
+      </c>
       <c r="F25" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="G25" s="18">
+      <c r="G25" s="5">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="H25" s="18">
+      <c r="H25" s="5">
         <v>4.5999999999999999E-2</v>
       </c>
-      <c r="I25" s="17">
-        <v>1</v>
-      </c>
-      <c r="J25" s="10"/>
+      <c r="I25" s="4">
+        <v>1</v>
+      </c>
       <c r="K25" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="L25" s="18">
+      <c r="L25" s="5">
         <v>3.7999999999999999E-2</v>
       </c>
-      <c r="M25" s="18">
+      <c r="M25" s="5">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="N25" s="17">
-        <v>1</v>
-      </c>
-      <c r="O25" s="10"/>
+      <c r="N25" s="4">
+        <v>1</v>
+      </c>
       <c r="P25" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="Q25" s="18">
+      <c r="Q25" s="5">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="R25" s="18">
+      <c r="R25" s="5">
         <v>0.05</v>
       </c>
-      <c r="S25" s="17">
-        <v>1</v>
-      </c>
-      <c r="T25" s="12"/>
+      <c r="S25" s="4">
+        <v>1</v>
+      </c>
+      <c r="T25" s="10"/>
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A26" s="15"/>
-      <c r="B26" s="10"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="10"/>
-      <c r="G26" s="10"/>
-      <c r="H26" s="10"/>
-      <c r="I26" s="10"/>
-      <c r="J26" s="10"/>
-      <c r="K26" s="10"/>
-      <c r="L26" s="10"/>
-      <c r="M26" s="10"/>
-      <c r="N26" s="10"/>
-      <c r="O26" s="10"/>
-      <c r="P26" s="10"/>
-      <c r="Q26" s="10"/>
-      <c r="R26" s="10"/>
-      <c r="S26" s="10"/>
-      <c r="T26" s="12"/>
+      <c r="A26" s="12"/>
+      <c r="T26" s="10"/>
     </row>
     <row r="27" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A27" s="15"/>
-      <c r="B27" s="10"/>
-      <c r="C27" s="10"/>
-      <c r="D27" s="10"/>
-      <c r="E27" s="10"/>
-      <c r="F27" s="10"/>
-      <c r="G27" s="10"/>
-      <c r="H27" s="10"/>
-      <c r="I27" s="10"/>
-      <c r="J27" s="10"/>
-      <c r="K27" s="10"/>
-      <c r="L27" s="10"/>
-      <c r="M27" s="10"/>
-      <c r="N27" s="10"/>
-      <c r="O27" s="10"/>
-      <c r="P27" s="10"/>
-      <c r="Q27" s="10"/>
-      <c r="R27" s="10"/>
-      <c r="S27" s="10"/>
-      <c r="T27" s="12"/>
+      <c r="A27" s="12"/>
+      <c r="T27" s="10"/>
     </row>
     <row r="28" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A28" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B28" s="10"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="10"/>
-      <c r="E28" s="10"/>
-      <c r="F28" s="11" t="s">
+      <c r="F28" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G28" s="10"/>
-      <c r="H28" s="10"/>
-      <c r="I28" s="10"/>
-      <c r="J28" s="10"/>
-      <c r="K28" s="11" t="s">
+      <c r="K28" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="L28" s="10"/>
-      <c r="M28" s="10"/>
-      <c r="N28" s="10"/>
-      <c r="O28" s="10"/>
-      <c r="P28" s="11" t="s">
+      <c r="P28" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Q28" s="10"/>
-      <c r="R28" s="10"/>
-      <c r="S28" s="10"/>
-      <c r="T28" s="12"/>
+      <c r="T28" s="10"/>
     </row>
     <row r="29" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A29" s="13" t="s">
+      <c r="A29" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="B29" s="10"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
-      <c r="F29" s="14" t="s">
+      <c r="F29" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G29" s="10"/>
-      <c r="H29" s="10"/>
-      <c r="I29" s="10"/>
-      <c r="J29" s="10"/>
-      <c r="K29" s="14" t="s">
+      <c r="K29" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="L29" s="10"/>
-      <c r="M29" s="10"/>
-      <c r="N29" s="10"/>
-      <c r="O29" s="10"/>
-      <c r="P29" s="14" t="s">
+      <c r="P29" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="Q29" s="10"/>
-      <c r="R29" s="10"/>
-      <c r="S29" s="10"/>
-      <c r="T29" s="12"/>
+      <c r="T29" s="10"/>
     </row>
     <row r="30" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A30" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="B30" s="10"/>
-      <c r="C30" s="10"/>
-      <c r="D30" s="10"/>
-      <c r="E30" s="10"/>
-      <c r="F30" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="G30" s="10"/>
-      <c r="H30" s="10"/>
-      <c r="I30" s="10"/>
-      <c r="J30" s="10"/>
-      <c r="K30" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="L30" s="10"/>
-      <c r="M30" s="10"/>
-      <c r="N30" s="10"/>
-      <c r="O30" s="10"/>
-      <c r="P30" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="Q30" s="10"/>
-      <c r="R30" s="10"/>
-      <c r="S30" s="10"/>
-      <c r="T30" s="12"/>
+      <c r="F30" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K30" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="P30" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="T30" s="10"/>
     </row>
     <row r="31" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A31" s="15"/>
+      <c r="A31" s="12"/>
       <c r="B31" s="3" t="s">
         <v>0</v>
       </c>
@@ -1546,8 +1400,6 @@
       <c r="D31" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E31" s="10"/>
-      <c r="F31" s="10"/>
       <c r="G31" s="3" t="s">
         <v>0</v>
       </c>
@@ -1557,8 +1409,6 @@
       <c r="I31" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="J31" s="10"/>
-      <c r="K31" s="10"/>
       <c r="L31" s="3" t="s">
         <v>0</v>
       </c>
@@ -1568,8 +1418,6 @@
       <c r="N31" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="O31" s="10"/>
-      <c r="P31" s="10"/>
       <c r="Q31" s="3" t="s">
         <v>0</v>
       </c>
@@ -1579,191 +1427,182 @@
       <c r="S31" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="T31" s="12"/>
+      <c r="T31" s="10"/>
     </row>
     <row r="32" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A32" s="16" t="s">
-        <v>0</v>
-      </c>
-      <c r="B32" s="17">
-        <v>1</v>
-      </c>
-      <c r="C32" s="17">
+      <c r="A32" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B32" s="4">
+        <v>1</v>
+      </c>
+      <c r="C32" s="4">
         <v>0.69</v>
       </c>
-      <c r="D32" s="17">
+      <c r="D32" s="4">
         <v>0.69</v>
       </c>
-      <c r="E32" s="10"/>
       <c r="F32" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="G32" s="17">
-        <v>1</v>
-      </c>
-      <c r="H32" s="17">
+      <c r="G32" s="4">
+        <v>1</v>
+      </c>
+      <c r="H32" s="4">
         <v>0.436</v>
       </c>
-      <c r="I32" s="18">
+      <c r="I32" s="5">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="J32" s="10"/>
       <c r="K32" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="L32" s="17">
-        <v>1</v>
-      </c>
-      <c r="M32" s="17">
+      <c r="L32" s="4">
+        <v>1</v>
+      </c>
+      <c r="M32" s="4">
         <v>0.52300000000000002</v>
       </c>
-      <c r="N32" s="18">
+      <c r="N32" s="5">
         <v>2.9000000000000001E-2</v>
       </c>
-      <c r="O32" s="10"/>
       <c r="P32" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="Q32" s="17">
-        <v>1</v>
-      </c>
-      <c r="R32" s="17">
+      <c r="Q32" s="4">
+        <v>1</v>
+      </c>
+      <c r="R32" s="4">
         <v>0.56999999999999995</v>
       </c>
-      <c r="S32" s="18">
+      <c r="S32" s="5">
         <v>0.01</v>
       </c>
-      <c r="T32" s="12"/>
+      <c r="T32" s="10"/>
     </row>
     <row r="33" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A33" s="16" t="s">
-        <v>1</v>
-      </c>
-      <c r="B33" s="17">
+      <c r="A33" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="B33" s="4">
         <v>0.69</v>
       </c>
-      <c r="C33" s="17">
-        <v>1</v>
-      </c>
-      <c r="D33" s="17">
+      <c r="C33" s="4">
+        <v>1</v>
+      </c>
+      <c r="D33" s="4">
         <v>0.69</v>
       </c>
-      <c r="E33" s="10"/>
       <c r="F33" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="G33" s="17">
+      <c r="G33" s="4">
         <v>0.436</v>
       </c>
-      <c r="H33" s="17">
-        <v>1</v>
-      </c>
-      <c r="I33" s="18">
+      <c r="H33" s="4">
+        <v>1</v>
+      </c>
+      <c r="I33" s="5">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="J33" s="10"/>
       <c r="K33" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="L33" s="17">
+      <c r="L33" s="4">
         <v>0.52300000000000002</v>
       </c>
-      <c r="M33" s="17">
-        <v>1</v>
-      </c>
-      <c r="N33" s="18">
+      <c r="M33" s="4">
+        <v>1</v>
+      </c>
+      <c r="N33" s="5">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="O33" s="10"/>
       <c r="P33" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="Q33" s="17">
+      <c r="Q33" s="4">
         <v>0.56999999999999995</v>
       </c>
-      <c r="R33" s="17">
-        <v>1</v>
-      </c>
-      <c r="S33" s="18">
+      <c r="R33" s="4">
+        <v>1</v>
+      </c>
+      <c r="S33" s="5">
         <v>2.5999999999999999E-2</v>
       </c>
-      <c r="T33" s="12"/>
+      <c r="T33" s="10"/>
     </row>
     <row r="34" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A34" s="16" t="s">
-        <v>2</v>
-      </c>
-      <c r="B34" s="17">
+      <c r="A34" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B34" s="4">
         <v>0.69</v>
       </c>
-      <c r="C34" s="17">
+      <c r="C34" s="4">
         <v>0.69</v>
       </c>
-      <c r="D34" s="17">
-        <v>1</v>
-      </c>
-      <c r="E34" s="10"/>
+      <c r="D34" s="4">
+        <v>1</v>
+      </c>
       <c r="F34" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="G34" s="18">
+      <c r="G34" s="5">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="H34" s="18">
+      <c r="H34" s="5">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="I34" s="17">
-        <v>1</v>
-      </c>
-      <c r="J34" s="10"/>
+      <c r="I34" s="4">
+        <v>1</v>
+      </c>
       <c r="K34" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="L34" s="18">
+      <c r="L34" s="5">
         <v>2.9000000000000001E-2</v>
       </c>
-      <c r="M34" s="18">
+      <c r="M34" s="5">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="N34" s="17">
-        <v>1</v>
-      </c>
-      <c r="O34" s="10"/>
+      <c r="N34" s="4">
+        <v>1</v>
+      </c>
       <c r="P34" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="Q34" s="18">
+      <c r="Q34" s="5">
         <v>0.01</v>
       </c>
-      <c r="R34" s="18">
+      <c r="R34" s="5">
         <v>2.5999999999999999E-2</v>
       </c>
-      <c r="S34" s="17">
-        <v>1</v>
-      </c>
-      <c r="T34" s="12"/>
+      <c r="S34" s="4">
+        <v>1</v>
+      </c>
+      <c r="T34" s="10"/>
     </row>
     <row r="35" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="19"/>
-      <c r="B35" s="20"/>
-      <c r="C35" s="20"/>
-      <c r="D35" s="20"/>
-      <c r="E35" s="20"/>
-      <c r="F35" s="20"/>
-      <c r="G35" s="20"/>
-      <c r="H35" s="20"/>
-      <c r="I35" s="20"/>
-      <c r="J35" s="20"/>
-      <c r="K35" s="20"/>
-      <c r="L35" s="20"/>
-      <c r="M35" s="20"/>
-      <c r="N35" s="20"/>
-      <c r="O35" s="20"/>
-      <c r="P35" s="20"/>
-      <c r="Q35" s="20"/>
-      <c r="R35" s="20"/>
-      <c r="S35" s="20"/>
-      <c r="T35" s="21"/>
+      <c r="A35" s="14"/>
+      <c r="B35" s="15"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="15"/>
+      <c r="H35" s="15"/>
+      <c r="I35" s="15"/>
+      <c r="J35" s="15"/>
+      <c r="K35" s="15"/>
+      <c r="L35" s="15"/>
+      <c r="M35" s="15"/>
+      <c r="N35" s="15"/>
+      <c r="O35" s="15"/>
+      <c r="P35" s="15"/>
+      <c r="Q35" s="15"/>
+      <c r="R35" s="15"/>
+      <c r="S35" s="15"/>
+      <c r="T35" s="16"/>
     </row>
     <row r="37" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">

</xml_diff>

<commit_message>
removed unnessesary files and added plot photoes
</commit_message>
<xml_diff>
--- a/Data/KW_dunn_between_month.xlsx
+++ b/Data/KW_dunn_between_month.xlsx
@@ -28,7 +28,7 @@
     <t>Group is wistar</t>
   </si>
   <si>
-    <t>Kruskal p-value for hyperplasia: 0.120</t>
+    <t>Kruskal p-value for hyperplasia: 0.978</t>
   </si>
   <si>
     <t>Dunn's post-hoc values with FDR-BH:</t>
@@ -67,7 +67,7 @@
     <t>Group is black</t>
   </si>
   <si>
-    <t>Kruskal p-value for hyperplasia: 0.033</t>
+    <t>Kruskal p-value for hyperplasia: 0.039</t>
   </si>
   <si>
     <t>Kruskal p-value for inflammation: 0.009</t>
@@ -573,10 +573,10 @@
         <v>1</v>
       </c>
       <c r="C5" s="4">
-        <v>0.164</v>
+        <v>0.915</v>
       </c>
       <c r="D5" s="4">
-        <v>0.164</v>
+        <v>0.915</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>0</v>
@@ -597,10 +597,10 @@
         <v>1</v>
       </c>
       <c r="M5" s="4">
-        <v>0.722</v>
+        <v>0.697</v>
       </c>
       <c r="N5" s="4">
-        <v>0.059</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="P5" s="3" t="s">
         <v>0</v>
@@ -609,7 +609,7 @@
         <v>1</v>
       </c>
       <c r="R5" s="4">
-        <v>0.288</v>
+        <v>0.289</v>
       </c>
       <c r="S5" s="5">
         <v>0.051</v>
@@ -620,13 +620,13 @@
         <v>1</v>
       </c>
       <c r="B6" s="4">
-        <v>0.164</v>
+        <v>0.915</v>
       </c>
       <c r="C6" s="4">
         <v>1</v>
       </c>
       <c r="D6" s="4">
-        <v>0.749</v>
+        <v>0.915</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>1</v>
@@ -644,19 +644,19 @@
         <v>1</v>
       </c>
       <c r="L6" s="4">
-        <v>0.722</v>
+        <v>0.697</v>
       </c>
       <c r="M6" s="4">
         <v>1</v>
       </c>
       <c r="N6" s="5">
-        <v>0.047</v>
+        <v>0.053</v>
       </c>
       <c r="P6" s="3" t="s">
         <v>1</v>
       </c>
       <c r="Q6" s="4">
-        <v>0.288</v>
+        <v>0.289</v>
       </c>
       <c r="R6" s="4">
         <v>1</v>
@@ -670,10 +670,10 @@
         <v>2</v>
       </c>
       <c r="B7" s="4">
-        <v>0.164</v>
+        <v>0.915</v>
       </c>
       <c r="C7" s="4">
-        <v>0.749</v>
+        <v>0.915</v>
       </c>
       <c r="D7" s="4">
         <v>1</v>
@@ -694,10 +694,10 @@
         <v>2</v>
       </c>
       <c r="L7" s="4">
-        <v>0.059</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="M7" s="5">
-        <v>0.047</v>
+        <v>0.053</v>
       </c>
       <c r="N7" s="4">
         <v>1</v>

</xml_diff>